<commit_message>
Update REGISTO VALORES NO COFRE EXCEL.xlsx
</commit_message>
<xml_diff>
--- a/REGISTO VALORES NO COFRE EXCEL.xlsx
+++ b/REGISTO VALORES NO COFRE EXCEL.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mythicsana-my.sharepoint.com/personal/info_downtownsuites_mythic_sanahotels_com/Documents/Night Auditor/Aplicação/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mythicsana-my.sharepoint.com/personal/info_downtownsuites_mythic_sanahotels_com/Documents/Night Auditor/FECHOS DO DIA 2026/Templates diários/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="251" documentId="11_9CD7481080C4552A941F5A76C504E9503659EA23" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E28DFA2-4B86-4BE0-A610-CC115C68CE0D}"/>
+  <xr:revisionPtr revIDLastSave="338" documentId="11_9CD7481080C4552A941F5A76C504E9503659EA23" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AB37375-7BA5-4FE6-A0C3-C704076ABFF7}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15943" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15943" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Table 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Valores" sheetId="1" r:id="rId1"/>
+    <sheet name="Envelope" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
   <si>
     <t>GASTROBAR</t>
   </si>
@@ -100,9 +101,6 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>DATA</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -152,6 +150,39 @@
   </si>
   <si>
     <t>Depósito de Valores no Cofre                                     05/04/2026</t>
+  </si>
+  <si>
+    <t>Maurílio Jr.</t>
+  </si>
+  <si>
+    <t>DATA:</t>
+  </si>
+  <si>
+    <t>DEPÓSITO:</t>
+  </si>
+  <si>
+    <t>F.O</t>
+  </si>
+  <si>
+    <t>F&amp;B</t>
+  </si>
+  <si>
+    <t>TOTAL:</t>
+  </si>
+  <si>
+    <t>PAIDOUTS:</t>
+  </si>
+  <si>
+    <t>OBSERVAÇÕES:</t>
+  </si>
+  <si>
+    <t>ASSINATURA:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEPÓSITO DO DIA: </t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
   <si>
     <r>
@@ -195,7 +226,8 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">
-TESTEMUNHA: -</t>
+TESTEMUNHA: GUILHERME ALVARENGA
+</t>
     </r>
   </si>
 </sst>
@@ -203,10 +235,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -284,6 +317,32 @@
       <b/>
       <sz val="9.5"/>
       <color rgb="FF3E3E3E"/>
+      <name val="Gill Sans Nova Light"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Gill Sans Nova Light"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Gill Sans Nova Light"/>
       <family val="2"/>
     </font>
@@ -302,12 +361,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor theme="1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -479,11 +538,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -499,9 +585,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -523,9 +606,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -535,23 +615,68 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="8" fontId="16" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="41"/>
@@ -562,15 +687,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="41"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="16"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="16"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="16"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -589,8 +705,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="12"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -610,8 +733,8 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>500743</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
@@ -643,7 +766,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
+          <a:off x="3303814" y="0"/>
           <a:ext cx="3743325" cy="814388"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -653,6 +776,61 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>146957</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>478971</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>27525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C6F0E87-5958-4D6E-9DAC-8217599919F2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3739243" y="0"/>
+          <a:ext cx="1899557" cy="631682"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -946,55 +1124,56 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13.3" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" style="18" customWidth="1"/>
-    <col min="2" max="2" width="22" style="18" customWidth="1"/>
-    <col min="3" max="3" width="25.36328125" style="18" customWidth="1"/>
-    <col min="4" max="4" width="24.1796875" style="18" customWidth="1"/>
-    <col min="5" max="5" width="22.453125" style="18" customWidth="1"/>
-    <col min="6" max="16384" width="9.1796875" style="18"/>
+    <col min="1" max="1" width="24.81640625" style="15" customWidth="1"/>
+    <col min="2" max="2" width="22" style="15" customWidth="1"/>
+    <col min="3" max="3" width="25.36328125" style="15" customWidth="1"/>
+    <col min="4" max="4" width="24.1796875" style="15" customWidth="1"/>
+    <col min="5" max="5" width="22.453125" style="15" customWidth="1"/>
+    <col min="6" max="16384" width="9.1796875" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="66.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="38"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="40"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="30">
+        <f ca="1">TODAY()-1</f>
+        <v>46193</v>
+      </c>
+      <c r="D2" s="28"/>
+      <c r="E2" s="29"/>
+    </row>
+    <row r="3" spans="1:5" ht="10.1" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="41"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="43"/>
+    </row>
+    <row r="4" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="16"/>
+      <c r="B4" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="25"/>
-    </row>
-    <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="28"/>
-    </row>
-    <row r="3" spans="1:5" ht="10.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="31"/>
-    </row>
-    <row r="4" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="19"/>
-      <c r="B4" s="20" t="s">
+      <c r="C4" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="D4" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="E4" s="19" t="s">
         <v>14</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
@@ -1004,161 +1183,406 @@
       <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="9">
         <v>0</v>
       </c>
       <c r="D5" s="3"/>
-      <c r="E5" s="9"/>
+      <c r="E5" s="8"/>
     </row>
     <row r="6" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4"/>
       <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>0</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="14"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="12"/>
     </row>
     <row r="7" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4"/>
       <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>0</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="8" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="4"/>
-      <c r="B8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="10">
+      <c r="E7" s="11"/>
+    </row>
+    <row r="8" spans="1:5" ht="6.55" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="31"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="35"/>
+    </row>
+    <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="9"/>
-    </row>
-    <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="4"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="13"/>
+      <c r="B9" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="9">
+        <v>0</v>
+      </c>
       <c r="D9" s="3"/>
-      <c r="E9" s="9"/>
+      <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="3"/>
+      <c r="B10" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="9">
         <v>0</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="10">
-        <v>0</v>
-      </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="9"/>
+      <c r="E10" s="12"/>
     </row>
     <row r="11" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="3"/>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="9">
+        <v>10</v>
+      </c>
+      <c r="D11" s="13"/>
+      <c r="E11" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="6.55" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="34"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="36"/>
+    </row>
+    <row r="13" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="9">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="8"/>
+    </row>
+    <row r="14" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="3"/>
+      <c r="B14" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C14" s="9">
         <v>0</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="14"/>
-    </row>
-    <row r="12" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="3"/>
-      <c r="B12" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12" s="10">
-        <v>0</v>
-      </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="14"/>
-    </row>
-    <row r="13" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="3"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="14"/>
-    </row>
-    <row r="14" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C14" s="10">
-        <v>0</v>
-      </c>
       <c r="D14" s="3"/>
-      <c r="E14" s="9"/>
+      <c r="E14" s="8"/>
     </row>
     <row r="15" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="3"/>
-      <c r="B15" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" s="10">
+      <c r="B15" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="9">
         <v>0</v>
       </c>
       <c r="D15" s="3"/>
-      <c r="E15" s="9"/>
+      <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="3"/>
-      <c r="B16" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" s="10">
-        <v>0</v>
+      <c r="A16" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="9">
+        <f>SUM(C5:C15)</f>
+        <v>10</v>
       </c>
       <c r="D16" s="3"/>
-      <c r="E16" s="9"/>
-    </row>
-    <row r="17" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="10">
-        <f>SUM(C5:C16)</f>
-        <v>0</v>
-      </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:5" ht="88.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="33"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="34"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5" ht="88.1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A2:B2"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="93" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33F156DC-8975-49E7-B41C-827713C51598}">
+  <dimension ref="A1:M16"/>
+  <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="21">
+        <f ca="1">Valores!C2</f>
+        <v>46193</v>
+      </c>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+    </row>
+    <row r="2" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+    </row>
+    <row r="3" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A3" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+    </row>
+    <row r="4" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A4" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="24">
+        <f>SUM(Valores!C5:C7)</f>
+        <v>0</v>
+      </c>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+    </row>
+    <row r="5" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A5" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="24">
+        <f>Valores!C11</f>
+        <v>10</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+    </row>
+    <row r="6" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A6" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="24">
+        <f>Valores!C16</f>
+        <v>10</v>
+      </c>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+    </row>
+    <row r="7" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A7" s="15"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
+    </row>
+    <row r="8" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A8" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="23">
+        <v>0</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+    </row>
+    <row r="9" spans="1:13" ht="15" x14ac:dyDescent="0.45">
+      <c r="A9" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="27">
+        <f>B6-B8</f>
+        <v>10</v>
+      </c>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+    </row>
+    <row r="10" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+    </row>
+    <row r="11" spans="1:13" ht="13.3" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
+      <c r="E11" s="37"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="37"/>
+      <c r="I11" s="37"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
+    </row>
+    <row r="12" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A12" s="15"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+    </row>
+    <row r="13" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A13" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+      <c r="L13" s="15"/>
+      <c r="M13" s="15"/>
+    </row>
+    <row r="16" spans="1:13" ht="14.15" x14ac:dyDescent="0.35">
+      <c r="B16" s="25"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B11:I12"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="27" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: improve auto-resize logic for text areas and trigger updates when switching to contagem tab
</commit_message>
<xml_diff>
--- a/REGISTO VALORES NO COFRE EXCEL.xlsx
+++ b/REGISTO VALORES NO COFRE EXCEL.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mythicsana-my.sharepoint.com/personal/info_downtownsuites_mythic_sanahotels_com/Documents/Night Auditor/Aplicação/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mythicsana-my.sharepoint.com/personal/info_downtownsuites_mythic_sanahotels_com/Documents/Night Auditor/FECHOS DO DIA 2026/Templates diários/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="251" documentId="11_9CD7481080C4552A941F5A76C504E9503659EA23" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E28DFA2-4B86-4BE0-A610-CC115C68CE0D}"/>
+  <xr:revisionPtr revIDLastSave="357" documentId="11_9CD7481080C4552A941F5A76C504E9503659EA23" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF605E80-45D3-4BBA-BF8C-7E47E8438473}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15943" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Table 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Valores" sheetId="1" r:id="rId1"/>
+    <sheet name="Envelope" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>GASTROBAR</t>
   </si>
@@ -100,9 +101,6 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>DATA</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -152,6 +150,36 @@
   </si>
   <si>
     <t>Depósito de Valores no Cofre                                     05/04/2026</t>
+  </si>
+  <si>
+    <t>DATA:</t>
+  </si>
+  <si>
+    <t>DEPÓSITO:</t>
+  </si>
+  <si>
+    <t>F.O</t>
+  </si>
+  <si>
+    <t>F&amp;B</t>
+  </si>
+  <si>
+    <t>TOTAL:</t>
+  </si>
+  <si>
+    <t>PAIDOUTS:</t>
+  </si>
+  <si>
+    <t>OBSERVAÇÕES:</t>
+  </si>
+  <si>
+    <t>ASSINATURA:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEPÓSITO DO DIA: </t>
+  </si>
+  <si>
+    <t>TOTAL RECEBIDO €233, VALOR UTILIZADO PARA ABATER PAIDOUTS REMANESCENTES NO TOTAL DE €11,90.</t>
   </si>
   <si>
     <r>
@@ -195,7 +223,8 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">
-TESTEMUNHA: -</t>
+TESTEMUNHA: JORGE DIAS
+TOTAL RECEBIDO €233, VALOR UTILIZADO PARA ABATER PAIDOUTS REMANESCENTES NO TOTAL DE €11,90.</t>
     </r>
   </si>
 </sst>
@@ -203,10 +232,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -284,6 +314,32 @@
       <b/>
       <sz val="9.5"/>
       <color rgb="FF3E3E3E"/>
+      <name val="Gill Sans Nova Light"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Gill Sans Nova Light"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Gill Sans Nova Light"/>
       <family val="2"/>
     </font>
@@ -302,12 +358,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor theme="1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -479,11 +535,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -499,9 +582,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -523,9 +603,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -535,23 +612,65 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="8" fontId="16" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="4"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="41"/>
@@ -562,15 +681,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="41"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="16"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="16"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="16"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -589,8 +699,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="12"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -610,10 +730,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>489857</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>16329</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3743325" cy="814388"/>
     <xdr:pic>
@@ -643,7 +763,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
+          <a:off x="3292928" y="16329"/>
           <a:ext cx="3743325" cy="814388"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -653,6 +773,61 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>146957</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>478971</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>27525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C6F0E87-5958-4D6E-9DAC-8217599919F2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3739243" y="0"/>
+          <a:ext cx="1899557" cy="631682"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -946,55 +1121,56 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13.3" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" style="18" customWidth="1"/>
-    <col min="2" max="2" width="22" style="18" customWidth="1"/>
-    <col min="3" max="3" width="25.36328125" style="18" customWidth="1"/>
-    <col min="4" max="4" width="24.1796875" style="18" customWidth="1"/>
-    <col min="5" max="5" width="22.453125" style="18" customWidth="1"/>
-    <col min="6" max="16384" width="9.1796875" style="18"/>
+    <col min="1" max="1" width="24.81640625" style="15" customWidth="1"/>
+    <col min="2" max="2" width="22" style="15" customWidth="1"/>
+    <col min="3" max="3" width="25.36328125" style="15" customWidth="1"/>
+    <col min="4" max="4" width="24.1796875" style="15" customWidth="1"/>
+    <col min="5" max="5" width="22.453125" style="15" customWidth="1"/>
+    <col min="6" max="16384" width="9.1796875" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="66.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="37"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="39"/>
+    </row>
+    <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="47"/>
+      <c r="C2" s="30">
+        <f ca="1">TODAY()-1</f>
+        <v>46217</v>
+      </c>
+      <c r="D2" s="28"/>
+      <c r="E2" s="29"/>
+    </row>
+    <row r="3" spans="1:5" ht="10.1" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="40"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="42"/>
+    </row>
+    <row r="4" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="16"/>
+      <c r="B4" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="25"/>
-    </row>
-    <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="28"/>
-    </row>
-    <row r="3" spans="1:5" ht="10.1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="29"/>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="31"/>
-    </row>
-    <row r="4" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="19"/>
-      <c r="B4" s="20" t="s">
+      <c r="C4" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="D4" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="E4" s="19" t="s">
         <v>14</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
@@ -1004,161 +1180,404 @@
       <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="10">
-        <v>0</v>
+      <c r="C5" s="9">
+        <v>221.1</v>
       </c>
       <c r="D5" s="3"/>
-      <c r="E5" s="9"/>
+      <c r="E5" s="8"/>
     </row>
     <row r="6" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4"/>
       <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>0</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="14"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="12"/>
     </row>
     <row r="7" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4"/>
       <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <v>0</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="8" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="4"/>
-      <c r="B8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="10">
+      <c r="E7" s="11"/>
+    </row>
+    <row r="8" spans="1:5" ht="6.55" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="31"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="35"/>
+    </row>
+    <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="9"/>
-    </row>
-    <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="4"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="13"/>
+      <c r="B9" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="9">
+        <v>0</v>
+      </c>
       <c r="D9" s="3"/>
-      <c r="E9" s="9"/>
+      <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="3"/>
+      <c r="B10" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="9">
         <v>0</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="10">
-        <v>0</v>
-      </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="9"/>
+      <c r="E10" s="12"/>
     </row>
     <row r="11" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="3"/>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="9">
+        <v>0</v>
+      </c>
+      <c r="D11" s="13"/>
+      <c r="E11" s="12"/>
+    </row>
+    <row r="12" spans="1:5" ht="6.55" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="34"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="36"/>
+    </row>
+    <row r="13" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="9">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="8"/>
+    </row>
+    <row r="14" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="3"/>
+      <c r="B14" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C14" s="9">
         <v>0</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="14"/>
-    </row>
-    <row r="12" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="3"/>
-      <c r="B12" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12" s="10">
-        <v>0</v>
-      </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="14"/>
-    </row>
-    <row r="13" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="3"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="14"/>
-    </row>
-    <row r="14" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C14" s="10">
-        <v>0</v>
-      </c>
       <c r="D14" s="3"/>
-      <c r="E14" s="9"/>
+      <c r="E14" s="8"/>
     </row>
     <row r="15" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="3"/>
-      <c r="B15" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" s="10">
+      <c r="B15" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="9">
         <v>0</v>
       </c>
       <c r="D15" s="3"/>
-      <c r="E15" s="9"/>
+      <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="3"/>
-      <c r="B16" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" s="10">
-        <v>0</v>
+      <c r="A16" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="9">
+        <f>SUM(C5:C15)</f>
+        <v>221.1</v>
       </c>
       <c r="D16" s="3"/>
-      <c r="E16" s="9"/>
-    </row>
-    <row r="17" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="10">
-        <f>SUM(C5:C16)</f>
-        <v>0</v>
-      </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:5" ht="88.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="33"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="34"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" spans="1:5" ht="88.1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="44"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A2:B2"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="93" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33F156DC-8975-49E7-B41C-827713C51598}">
+  <dimension ref="A1:M16"/>
+  <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="21">
+        <f ca="1">Valores!C2</f>
+        <v>46217</v>
+      </c>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+    </row>
+    <row r="2" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+    </row>
+    <row r="3" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A3" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+    </row>
+    <row r="4" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A4" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="24">
+        <f>SUM(Valores!C5:C7)</f>
+        <v>221.1</v>
+      </c>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+    </row>
+    <row r="5" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A5" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="24">
+        <f>Valores!C11</f>
+        <v>0</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+    </row>
+    <row r="6" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A6" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="24">
+        <f>Valores!C16</f>
+        <v>221.1</v>
+      </c>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+    </row>
+    <row r="7" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A7" s="15"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
+    </row>
+    <row r="8" spans="1:13" ht="13.3" x14ac:dyDescent="0.4">
+      <c r="A8" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="23">
+        <v>0</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+    </row>
+    <row r="9" spans="1:13" ht="15" x14ac:dyDescent="0.45">
+      <c r="A9" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="27">
+        <f>B6-B8</f>
+        <v>221.1</v>
+      </c>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+    </row>
+    <row r="10" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+    </row>
+    <row r="11" spans="1:13" ht="13.3" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
+      <c r="H11" s="48"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
+    </row>
+    <row r="12" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A12" s="15"/>
+      <c r="B12" s="48"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
+      <c r="H12" s="48"/>
+      <c r="I12" s="48"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+    </row>
+    <row r="13" spans="1:13" ht="13.3" x14ac:dyDescent="0.35">
+      <c r="A13" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+      <c r="L13" s="15"/>
+      <c r="M13" s="15"/>
+    </row>
+    <row r="16" spans="1:13" ht="14.15" x14ac:dyDescent="0.35">
+      <c r="B16" s="25"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B11:I12"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="27" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>